<commit_message>
Updated the Cheat_Sheet_SecuritateIT file
s
</commit_message>
<xml_diff>
--- a/Cheat_Sheet_SecuritateIT.xlsx
+++ b/Cheat_Sheet_SecuritateIT.xlsx
@@ -72,7 +72,7 @@
     <t xml:space="preserve">Show all commits, starting wiht the newest</t>
   </si>
   <si>
-    <t xml:space="preserve">At the end of each day be sure to: git status and if everything ok git push</t>
+    <t xml:space="preserve">At the end of each day or training sesion be sure to: git status and if everything ok git push</t>
   </si>
 </sst>
 </file>
@@ -132,17 +132,17 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right/>
+      <right style="none"/>
       <top style="thin">
         <color auto="1"/>
       </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
     <border>
-      <left/>
+      <left style="none"/>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -152,7 +152,7 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">

</xml_diff>

<commit_message>
Updated the Cheat_Sheet_SecuritateIT.xlsx with some basic network commands in cmd
</commit_message>
<xml_diff>
--- a/Cheat_Sheet_SecuritateIT.xlsx
+++ b/Cheat_Sheet_SecuritateIT.xlsx
@@ -16,36 +16,69 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t xml:space="preserve">GitHub </t>
   </si>
   <si>
+    <t xml:space="preserve">Network Commands</t>
+  </si>
+  <si>
     <t>command</t>
   </si>
   <si>
+    <t xml:space="preserve">ping google.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pings the server and see the connectivity</t>
+  </si>
+  <si>
     <t xml:space="preserve">git init</t>
   </si>
   <si>
     <t xml:space="preserve">Create a new local repository</t>
   </si>
   <si>
+    <t>ipconfig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">it will display the network configuration</t>
+  </si>
+  <si>
     <t xml:space="preserve">git add .</t>
   </si>
   <si>
     <t xml:space="preserve">This adds all the current changes to the next commit</t>
   </si>
   <si>
+    <t xml:space="preserve">ipconfig /all</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Displays all the network configuration</t>
+  </si>
+  <si>
     <t xml:space="preserve">git commit -m "commit message"</t>
   </si>
   <si>
     <t xml:space="preserve">this will add a message to keep track of modification or added files</t>
   </si>
   <si>
+    <t xml:space="preserve">tracert google.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It will show all the hops that the packages are going</t>
+  </si>
+  <si>
     <t xml:space="preserve">git branch -M main</t>
   </si>
   <si>
     <t xml:space="preserve">Branch to main</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nslookup facebook.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It will display the ip of the facebook.com</t>
   </si>
   <si>
     <t xml:space="preserve">git remote add origin </t>
@@ -158,12 +191,15 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
@@ -635,6 +671,8 @@
   <cols>
     <col bestFit="1" min="1" max="1" width="29.140625"/>
     <col bestFit="1" min="2" max="2" width="56.7109375"/>
+    <col bestFit="1" min="3" max="3" width="32.140625"/>
+    <col bestFit="1" min="4" max="4" width="44.28125"/>
   </cols>
   <sheetData>
     <row r="1" ht="26.25">
@@ -642,83 +680,115 @@
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
       <c r="D1" s="2"/>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>11</v>
+        <v>21</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="5"/>
+      <c r="A11" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Updated the Cheat_Sheet_SecuritateIT.xlsx file with another option for git commit without -m
</commit_message>
<xml_diff>
--- a/Cheat_Sheet_SecuritateIT.xlsx
+++ b/Cheat_Sheet_SecuritateIT.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t xml:space="preserve">GitHub </t>
   </si>
@@ -106,6 +106,30 @@
   </si>
   <si>
     <t xml:space="preserve">At the end of each day or training sesion be sure to: git status and if everything ok git push</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Another way of commit a message is to use git add . git commit git push</t>
+  </si>
+  <si>
+    <t xml:space="preserve">on  the bash type the commit mesage and after that :qw </t>
+  </si>
+  <si>
+    <t>Esc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">:w -&gt; write/save</t>
+  </si>
+  <si>
+    <t xml:space="preserve">:q -&gt; quit</t>
+  </si>
+  <si>
+    <t>Enter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if you want to exit without commit</t>
+  </si>
+  <si>
+    <t>:q!</t>
   </si>
 </sst>
 </file>
@@ -191,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -209,6 +233,10 @@
     <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -790,9 +818,61 @@
       </c>
       <c r="B11" s="6"/>
     </row>
+    <row r="12" ht="14.25">
+      <c r="A12" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="7"/>
+    </row>
+    <row r="13" ht="14.25">
+      <c r="A13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" ht="14.25">
+      <c r="A14" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" ht="14.25">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" ht="14.25">
+      <c r="A16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" ht="14.25">
+      <c r="A17" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="A19" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="A20" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="A21" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="B7"/>

</xml_diff>

<commit_message>
update the M1_2_Retele&Internet.txt and also update Cheat_Sheet_SecuritateIT.xlxs file till OSI model Sheet.
</commit_message>
<xml_diff>
--- a/Cheat_Sheet_SecuritateIT.xlsx
+++ b/Cheat_Sheet_SecuritateIT.xlsx
@@ -3,10 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Various commands" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="IP Addresses" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Home and Corporate Network" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="OSI Model" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -16,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t xml:space="preserve">GitHub </t>
   </si>
@@ -130,6 +133,97 @@
   </si>
   <si>
     <t>:q!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IP address</t>
+  </si>
+  <si>
+    <t>192.168.1.0/24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Think of this as street Eminescu nr1 and the 192.168.1.0/24 and there will be a house with 256 rooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">this means that the above network can have 256 addresees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">from 192.168.1.0 till 192.168.1.255</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Think of this as street Eminescu nr2 and the 192.168.2.0/24 and there will be a house with 256 rooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if we have 192.168.2.0/24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This means that the above network is another one and can still have 256 addresses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">in an IP address the first and last address canot be dedicated to a device. 
+The 192.168.1.0 is the network address. 
+The 192.168.1.1 is the router addres and the 
+192.168.1.255 is the broadband address. 
+This means that the devices can have addresses from 192.168.1.2 till 192.168.1.254</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Private ip addresses</t>
+  </si>
+  <si>
+    <t>192.168.0.0</t>
+  </si>
+  <si>
+    <t>172.16.0.0</t>
+  </si>
+  <si>
+    <t>10.0.0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OSI Model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 layers</t>
+  </si>
+  <si>
+    <t>Application</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTP,HTTPS,
+FTP, DHCP,
+PNG</t>
+  </si>
+  <si>
+    <t>Presentation</t>
+  </si>
+  <si>
+    <t>Session</t>
+  </si>
+  <si>
+    <t>Transport</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TCP. UDP</t>
+  </si>
+  <si>
+    <t>Internet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IP, ARP, ICMP</t>
+  </si>
+  <si>
+    <t>Network</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WI-Fi
+Ethernet</t>
+  </si>
+  <si>
+    <t>Datalink</t>
+  </si>
+  <si>
+    <t>Physical</t>
   </si>
 </sst>
 </file>
@@ -162,7 +256,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="12">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -211,11 +305,91 @@
       </bottom>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="none"/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="none"/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="24">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -237,6 +411,51 @@
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="7" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="8" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="7" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="9" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="10" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="11" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -249,6 +468,73 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="6095999" cy="3596826"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="650506118" name=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm flipH="0" flipV="0">
+          <a:off x="0" y="0"/>
+          <a:ext cx="6095999" cy="3596826"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>361949</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="7067549" cy="5580042"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="434009817" name=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm flipH="0" flipV="0">
+          <a:off x="6457949" y="0"/>
+          <a:ext cx="7067549" cy="5580042"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
@@ -882,4 +1168,553 @@
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col bestFit="1" min="1" max="1" width="17.7109375"/>
+    <col customWidth="1" min="2" max="2" width="18.7109375"/>
+    <col customWidth="1" min="3" max="3" width="19.00390625"/>
+    <col customWidth="1" min="4" max="4" width="16.28125"/>
+    <col customWidth="1" min="5" max="5" width="21.00390625"/>
+    <col customWidth="1" min="10" max="10" width="14.57421875"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+    </row>
+    <row r="2">
+      <c r="B2" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+      <c r="N5" s="11"/>
+    </row>
+    <row r="6">
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+      <c r="N6" s="11"/>
+    </row>
+    <row r="7">
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
+      <c r="N7" s="11"/>
+    </row>
+    <row r="8">
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="11"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11"/>
+      <c r="M8" s="11"/>
+      <c r="N8" s="11"/>
+    </row>
+    <row r="9">
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="11"/>
+      <c r="N9" s="11"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:N1"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F3:N3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="F5:N9"/>
+  </mergeCells>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="N2" s="12"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="7"/>
+      <c r="J20" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J20"/>
+  </mergeCells>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="13.7109375"/>
+    <col customWidth="1" min="2" max="2" width="17.421875"/>
+    <col bestFit="1" min="3" max="3" width="11.7109375"/>
+    <col customWidth="1" min="4" max="4" width="5.57421875"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" s="16">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="18">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" s="18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" s="18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D12" s="23">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+  </mergeCells>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated the Cheat_Sheet_SecuritateIT.xlsx/OSI Model shet with a snipet of one of OSI model layer
</commit_message>
<xml_diff>
--- a/Cheat_Sheet_SecuritateIT.xlsx
+++ b/Cheat_Sheet_SecuritateIT.xlsx
@@ -526,6 +526,42 @@
         <a:xfrm flipH="0" flipV="0">
           <a:off x="6457949" y="0"/>
           <a:ext cx="7067549" cy="5580042"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>609599</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="11271521" cy="5619749"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="797999608" name=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm flipH="0" flipV="0">
+          <a:off x="4448174" y="0"/>
+          <a:ext cx="11271521" cy="5619749"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1619,6 +1655,9 @@
         <v>52</v>
       </c>
     </row>
+    <row r="2">
+      <c r="K2" s="12"/>
+    </row>
     <row r="6">
       <c r="A6" s="13" t="s">
         <v>53</v>
@@ -1716,5 +1755,6 @@
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Just finished the day with ARP on m1.2 module. I will update later or before the next session
</commit_message>
<xml_diff>
--- a/Cheat_Sheet_SecuritateIT.xlsx
+++ b/Cheat_Sheet_SecuritateIT.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="110">
   <si>
     <t xml:space="preserve">GitHub </t>
   </si>
@@ -189,7 +189,7 @@
   <si>
     <t xml:space="preserve">HTTP,HTTPS,
 FTP, DHCP,
-PNG</t>
+PNG, SSH, SMTP</t>
   </si>
   <si>
     <t>Presentation</t>
@@ -224,6 +224,184 @@
   </si>
   <si>
     <t>Physical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Layer 1 - Physical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Role: Transmits raw bits over a phisical medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Examples:
+Ethernet cable
+Fiber Optic cable
+Wi-Fi radio signals
+Connectors (RJ45)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Devices:
+Hub
+Repeater </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data units: Bits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simple explanation:
+Defines how electrical, light or radio signals travel between devices</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Layer 2 - Data Link</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Role: Transfers data between devices on the same LAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Examples:
+Ethernet
+Wi-Fi (802.11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Devices:
+Switch
+NIC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Addressing:
+MAC Address</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Unit: Frame</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simple explanation:
+Uses MAC addresses to ensure data reaches the correct device within local network</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Layer 3 - Network</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Role: Routes data between different networks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exmples:
+IP(IPv4, IPv6)
+ICMP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Devices:
+Router
+Layer 3 switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Addressing:
+IP Address</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Unit: Packet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simple explanation:
+Uses IP addresses to fid the best path and deliver data from a network to another</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Layer 4 - transport</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Role: provides end-to-end communication between applications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Examples:
+TCP
+UDP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functions:
+Segmentation
+Error checking
+Flow control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Addressing:
+Port numbers
+80,443,22...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data unit:
+Segment(TCP)
+Datagram(UDP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simple Explanation:
+Ensures data is delivered to the correct application and, with TCP, reliably and in the correct order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Layer 5 - Sesion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Role: Establishes, manages, and terminates communication sessions between applications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Examples:
+NetBIOS
+RPC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functions:
+Session creation
+Session maintenance
+Session termination</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Unit: Data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simple Exaplanation:
+Keeps track of conversation between two application and controls when a communication session starts and ends</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Layer 6 - Presentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Role: Translate, encryps and compresses data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Examples:
+SSL/TLS, JPEG,
+PNG, ASCII</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functions:
+Data Formating
+Encryption/Decryption
+Compression/Decompression</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simple Explanation:
+Ensures that data sent by one device can be correctly understood by the receiving device, regardles of differences in data format. It can also encrypt and decompress the data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Layer 7 - Application</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Role: provides network services directly to user applications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Examples:
+HTTP/HTTPS, DNS, 
+FTP, SMTP, SSH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functions:
+Web browsing, email, 
+file transfer, name resolution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data unit: Data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simple explanation:
+This is the layer cosest to the user. It allows applications such as web broesers, email clients and file transfer tools to communicate over the network</t>
   </si>
 </sst>
 </file>
@@ -389,7 +567,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="31">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -455,6 +633,27 @@
     </xf>
     <xf fontId="0" fillId="0" borderId="11" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -541,12 +740,12 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>609599</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>28574</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>76199</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="11271521" cy="5619749"/>
+    <xdr:ext cx="10480946" cy="5225585"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="797999608" name=""/>
@@ -560,8 +759,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm flipH="0" flipV="0">
-          <a:off x="4448174" y="0"/>
-          <a:ext cx="11271521" cy="5619749"/>
+          <a:off x="28574" y="7448549"/>
+          <a:ext cx="10480946" cy="5225585"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1639,15 +1838,18 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="13.7109375"/>
+    <col customWidth="1" min="1" max="1" width="19.7109375"/>
     <col customWidth="1" min="2" max="2" width="17.421875"/>
     <col bestFit="1" min="3" max="3" width="11.7109375"/>
     <col customWidth="1" min="4" max="4" width="5.57421875"/>
+    <col customWidth="1" min="5" max="5" width="23.57421875"/>
+    <col customWidth="1" min="8" max="8" width="28.7109375"/>
+    <col customWidth="1" min="9" max="9" width="14.00390625"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="14.25">
       <c r="A1" t="s">
         <v>51</v>
       </c>
@@ -1655,101 +1857,615 @@
         <v>52</v>
       </c>
     </row>
-    <row r="2">
-      <c r="K2" s="12"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="13" t="s">
+    <row r="3" ht="14.25">
+      <c r="A3" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B3" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C3" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="D6" s="16">
+      <c r="D3" s="16">
         <v>7</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="17"/>
-      <c r="B7" s="7"/>
+    <row r="4" ht="14.25">
+      <c r="A4" s="17"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="18">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" ht="14.25">
+      <c r="A5" s="17"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" ht="14.25">
+      <c r="A6" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25">
+      <c r="A7" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>60</v>
+      </c>
       <c r="C7" s="7" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D7" s="18">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="17"/>
-      <c r="B8" s="7"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" ht="14.25">
+      <c r="A8" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>63</v>
+      </c>
       <c r="C8" s="7" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D8" s="18">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="D9" s="18">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D10" s="18">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="B11" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="D11" s="18">
         <v>2</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="21"/>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22" t="s">
+    <row r="9" ht="14.25">
+      <c r="A9" s="21"/>
+      <c r="B9" s="22"/>
+      <c r="C9" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="D12" s="23">
+      <c r="D9" s="23">
         <v>1</v>
       </c>
     </row>
+    <row r="13" ht="14.25">
+      <c r="A13" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="G13" s="24"/>
+      <c r="H13" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="I13" s="11"/>
+      <c r="J13" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="K13" s="24"/>
+      <c r="L13" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="M13" s="26"/>
+      <c r="N13" s="26"/>
+      <c r="O13" s="26"/>
+      <c r="P13" s="26"/>
+    </row>
+    <row r="14" ht="14.25">
+      <c r="A14" s="24"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="24"/>
+      <c r="L14" s="26"/>
+      <c r="M14" s="26"/>
+      <c r="N14" s="26"/>
+      <c r="O14" s="26"/>
+      <c r="P14" s="26"/>
+    </row>
+    <row r="15" ht="14.25">
+      <c r="A15" s="24"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="24"/>
+      <c r="K15" s="24"/>
+      <c r="L15" s="26"/>
+      <c r="M15" s="26"/>
+      <c r="N15" s="26"/>
+      <c r="O15" s="26"/>
+      <c r="P15" s="26"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="24"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
+      <c r="L16" s="26"/>
+      <c r="M16" s="26"/>
+      <c r="N16" s="26"/>
+      <c r="O16" s="26"/>
+      <c r="P16" s="26"/>
+    </row>
+    <row r="17" ht="14.25">
+      <c r="A17" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" s="24" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="G17" s="11"/>
+      <c r="H17" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="J17" s="27" t="s">
+        <v>77</v>
+      </c>
+      <c r="K17" s="26"/>
+      <c r="L17" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="M17" s="26"/>
+      <c r="N17" s="26"/>
+      <c r="O17" s="26"/>
+      <c r="P17" s="26"/>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="A18" s="24"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="26"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="26"/>
+      <c r="K18" s="26"/>
+      <c r="L18" s="26"/>
+      <c r="M18" s="26"/>
+      <c r="N18" s="26"/>
+      <c r="O18" s="26"/>
+      <c r="P18" s="26"/>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="A19" s="24"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="26"/>
+      <c r="K19" s="26"/>
+      <c r="L19" s="26"/>
+      <c r="M19" s="26"/>
+      <c r="N19" s="26"/>
+      <c r="O19" s="26"/>
+      <c r="P19" s="26"/>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="A20" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" s="26"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="G20" s="26"/>
+      <c r="H20" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="I20" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="J20" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="K20" s="26"/>
+      <c r="L20" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="M20" s="26"/>
+      <c r="N20" s="26"/>
+      <c r="O20" s="26"/>
+      <c r="P20" s="26"/>
+    </row>
+    <row r="21" ht="31.5" customHeight="1">
+      <c r="A21" s="26"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="26"/>
+      <c r="K21" s="26"/>
+      <c r="L21" s="26"/>
+      <c r="M21" s="26"/>
+      <c r="N21" s="26"/>
+      <c r="O21" s="26"/>
+      <c r="P21" s="26"/>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="A22" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="G22" s="26"/>
+      <c r="H22" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="I22" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="J22" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="K22" s="26"/>
+      <c r="L22" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="M22" s="26"/>
+      <c r="N22" s="26"/>
+      <c r="O22" s="26"/>
+      <c r="P22" s="26"/>
+    </row>
+    <row r="23" ht="14.25">
+      <c r="A23" s="26"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="28"/>
+      <c r="I23" s="26"/>
+      <c r="J23" s="26"/>
+      <c r="K23" s="26"/>
+      <c r="L23" s="26"/>
+      <c r="M23" s="26"/>
+      <c r="N23" s="26"/>
+      <c r="O23" s="26"/>
+      <c r="P23" s="26"/>
+    </row>
+    <row r="24" ht="29.25" customHeight="1">
+      <c r="A24" s="26"/>
+      <c r="B24" s="26"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="28"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="26"/>
+      <c r="K24" s="26"/>
+      <c r="L24" s="26"/>
+      <c r="M24" s="26"/>
+      <c r="N24" s="26"/>
+      <c r="O24" s="26"/>
+      <c r="P24" s="26"/>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="A25" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="B25" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="G25" s="26"/>
+      <c r="H25" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="I25" s="26"/>
+      <c r="J25" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="K25" s="26"/>
+      <c r="L25" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="M25" s="26"/>
+      <c r="N25" s="26"/>
+      <c r="O25" s="26"/>
+      <c r="P25" s="26"/>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="A26" s="24"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="26"/>
+      <c r="H26" s="26"/>
+      <c r="I26" s="26"/>
+      <c r="J26" s="26"/>
+      <c r="K26" s="26"/>
+      <c r="L26" s="26"/>
+      <c r="M26" s="26"/>
+      <c r="N26" s="26"/>
+      <c r="O26" s="26"/>
+      <c r="P26" s="26"/>
+    </row>
+    <row r="27" ht="29.25" customHeight="1">
+      <c r="A27" s="24"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="26"/>
+      <c r="I27" s="26"/>
+      <c r="J27" s="26"/>
+      <c r="K27" s="26"/>
+      <c r="L27" s="26"/>
+      <c r="M27" s="26"/>
+      <c r="N27" s="26"/>
+      <c r="O27" s="26"/>
+      <c r="P27" s="26"/>
+    </row>
+    <row r="28" ht="14.25">
+      <c r="A28" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="B28" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="G28" s="26"/>
+      <c r="H28" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="I28" s="26"/>
+      <c r="J28" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="K28" s="26"/>
+      <c r="L28" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="M28" s="26"/>
+      <c r="N28" s="26"/>
+      <c r="O28" s="26"/>
+      <c r="P28" s="26"/>
+    </row>
+    <row r="29" ht="14.25">
+      <c r="A29" s="24"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="26"/>
+      <c r="H29" s="26"/>
+      <c r="I29" s="26"/>
+      <c r="J29" s="26"/>
+      <c r="K29" s="26"/>
+      <c r="L29" s="26"/>
+      <c r="M29" s="26"/>
+      <c r="N29" s="26"/>
+      <c r="O29" s="26"/>
+      <c r="P29" s="26"/>
+    </row>
+    <row r="30" ht="47.25" customHeight="1">
+      <c r="A30" s="24"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="26"/>
+      <c r="L30" s="26"/>
+      <c r="M30" s="26"/>
+      <c r="N30" s="26"/>
+      <c r="O30" s="26"/>
+      <c r="P30" s="26"/>
+    </row>
+    <row r="31" ht="14.25">
+      <c r="A31" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="B31" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="C31" s="26"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="G31" s="26"/>
+      <c r="H31" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="I31" s="24"/>
+      <c r="J31" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="K31" s="30"/>
+      <c r="L31" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="M31" s="26"/>
+      <c r="N31" s="26"/>
+      <c r="O31" s="26"/>
+      <c r="P31" s="26"/>
+    </row>
+    <row r="32" ht="14.25">
+      <c r="A32" s="26"/>
+      <c r="B32" s="26"/>
+      <c r="C32" s="26"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="26"/>
+      <c r="G32" s="26"/>
+      <c r="H32" s="26"/>
+      <c r="I32" s="24"/>
+      <c r="J32" s="30"/>
+      <c r="K32" s="30"/>
+      <c r="L32" s="26"/>
+      <c r="M32" s="26"/>
+      <c r="N32" s="26"/>
+      <c r="O32" s="26"/>
+      <c r="P32" s="26"/>
+    </row>
+    <row r="33" ht="35.25" customHeight="1">
+      <c r="A33" s="26"/>
+      <c r="B33" s="26"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="26"/>
+      <c r="F33" s="26"/>
+      <c r="G33" s="26"/>
+      <c r="H33" s="26"/>
+      <c r="I33" s="24"/>
+      <c r="J33" s="30"/>
+      <c r="K33" s="30"/>
+      <c r="L33" s="26"/>
+      <c r="M33" s="26"/>
+      <c r="N33" s="26"/>
+      <c r="O33" s="26"/>
+      <c r="P33" s="26"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
+  <mergeCells count="53">
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="B13:E16"/>
+    <mergeCell ref="F13:G16"/>
+    <mergeCell ref="H13:H16"/>
+    <mergeCell ref="I13:I16"/>
+    <mergeCell ref="J13:K16"/>
+    <mergeCell ref="L13:P16"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="B17:E19"/>
+    <mergeCell ref="F17:G19"/>
+    <mergeCell ref="H17:H19"/>
+    <mergeCell ref="I17:I19"/>
+    <mergeCell ref="J17:K19"/>
+    <mergeCell ref="L17:P19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:E21"/>
+    <mergeCell ref="F20:G21"/>
+    <mergeCell ref="H20:H21"/>
+    <mergeCell ref="I20:I21"/>
+    <mergeCell ref="J20:K21"/>
+    <mergeCell ref="L20:P21"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="B22:E24"/>
+    <mergeCell ref="F22:G24"/>
+    <mergeCell ref="H22:H24"/>
+    <mergeCell ref="I22:I24"/>
+    <mergeCell ref="J22:K24"/>
+    <mergeCell ref="L22:P24"/>
+    <mergeCell ref="A25:A27"/>
+    <mergeCell ref="B25:E27"/>
+    <mergeCell ref="F25:G27"/>
+    <mergeCell ref="H25:H27"/>
+    <mergeCell ref="I25:I27"/>
+    <mergeCell ref="J25:K27"/>
+    <mergeCell ref="L25:P27"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="B28:E30"/>
+    <mergeCell ref="F28:G30"/>
+    <mergeCell ref="H28:H30"/>
+    <mergeCell ref="I28:I30"/>
+    <mergeCell ref="J28:K30"/>
+    <mergeCell ref="L28:P30"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="B31:E33"/>
+    <mergeCell ref="F31:G33"/>
+    <mergeCell ref="H31:H33"/>
+    <mergeCell ref="I31:I33"/>
+    <mergeCell ref="J31:K33"/>
+    <mergeCell ref="L31:P33"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Almost finished with M2 module. Added some basic commands lab and a static routing lab. updated the Cheat_Sheet file
</commit_message>
<xml_diff>
--- a/Cheat_Sheet_SecuritateIT.xlsx
+++ b/Cheat_Sheet_SecuritateIT.xlsx
@@ -3,13 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Various commands" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="IP Addresses" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Home and Corporate Network" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="OSI Model" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CISCO PACKET TRACER" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="152">
   <si>
     <t xml:space="preserve">GitHub </t>
   </si>
@@ -403,12 +404,138 @@
     <t xml:space="preserve">Simple explanation:
 This is the layer cosest to the user. It allows applications such as web broesers, email clients and file transfer tools to communicate over the network</t>
   </si>
+  <si>
+    <t xml:space="preserve">CISCO PACKET TRACER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Common commands </t>
+  </si>
+  <si>
+    <t>explanation</t>
+  </si>
+  <si>
+    <t>example:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enable </t>
+  </si>
+  <si>
+    <t xml:space="preserve">turn on priviledged mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">configure terminal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter global configuration mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">show ip interface brief</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Display all interfaces and their status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">interface </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Select a interface to configure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">interface Gig0/0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ip address</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assign an ip address to an interface</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ip address 192.168.0.1 255.255.255.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no shutdown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enable (activate) the interface</t>
+  </si>
+  <si>
+    <t>iproute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add a static route</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ip route 192.168.0.0 255.255.255.0 192.168.1.1</t>
+  </si>
+  <si>
+    <t>hostname</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set the device name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enable password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set priviledged mode password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enable password admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enable secret</t>
+  </si>
+  <si>
+    <t xml:space="preserve">set an encrypted priviledged mode password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">banner motd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set a message for unauthorized users</t>
+  </si>
+  <si>
+    <t xml:space="preserve">banner motd "Access denied for unauthorized users"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Telnet configure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1(config)#line vty 0 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">allows up to 5 simulatenous connections</t>
+  </si>
+  <si>
+    <t xml:space="preserve">line vty 0 2 -allows 3 simutaneous connection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1(config-line)#password </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provides a password for telnet connection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">password admin</t>
+  </si>
+  <si>
+    <t>R1(config-line)#login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Starts the authentification with telnet</t>
+  </si>
+  <si>
+    <t>login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSH config</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11.000000"/>
       <name val="Calibri"/>
@@ -424,6 +551,11 @@
       <sz val="11.000000"/>
       <color theme="10"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="12.000000"/>
+      <color indexed="64"/>
+      <name val="Times New Roman"/>
     </font>
   </fonts>
   <fills count="2">
@@ -567,7 +699,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="28">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -589,12 +721,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -619,9 +745,6 @@
     <xf fontId="0" fillId="0" borderId="8" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="7" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -637,23 +760,19 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -678,7 +797,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="6095999" cy="3596826"/>
+    <xdr:ext cx="6095998" cy="3596825"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="650506118" name=""/>
@@ -705,11 +824,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>361949</xdr:colOff>
+      <xdr:colOff>361948</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="7067549" cy="5580042"/>
+    <xdr:ext cx="7067549" cy="5580041"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="434009817" name=""/>
@@ -1218,10 +1337,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr baseColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col bestFit="1" min="1" max="1" width="29.140625"/>
+    <col customWidth="1" min="1" max="1" width="30.57421875"/>
     <col bestFit="1" min="2" max="2" width="56.7109375"/>
     <col bestFit="1" min="3" max="3" width="32.140625"/>
     <col bestFit="1" min="4" max="4" width="44.28125"/>
+    <col customWidth="1" min="5" max="5" width="25.421875"/>
   </cols>
   <sheetData>
     <row r="1" ht="26.25">
@@ -1421,26 +1541,26 @@
       <c r="A1" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="7" t="s">
         <v>39</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
       <c r="E1" s="7"/>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
     </row>
     <row r="2">
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="7" t="s">
         <v>41</v>
       </c>
       <c r="C2" s="7"/>
@@ -1453,13 +1573,13 @@
       <c r="J2" s="7"/>
     </row>
     <row r="3">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="7" t="s">
         <v>42</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="7" t="s">
         <v>43</v>
       </c>
       <c r="G3" s="7"/>
@@ -1472,7 +1592,7 @@
       <c r="N3" s="7"/>
     </row>
     <row r="4">
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="7" t="s">
         <v>44</v>
       </c>
       <c r="C4" s="7"/>
@@ -1480,67 +1600,67 @@
       <c r="E4" s="7"/>
     </row>
     <row r="5">
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="7" t="s">
         <v>45</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
     </row>
     <row r="6">
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
     </row>
     <row r="7">
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
     </row>
     <row r="8">
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="11"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
     </row>
     <row r="9">
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
@@ -1606,7 +1726,7 @@
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
-      <c r="N2" s="12"/>
+      <c r="N2" s="10"/>
     </row>
     <row r="3">
       <c r="A3" s="7"/>
@@ -1858,41 +1978,41 @@
       </c>
     </row>
     <row r="3" ht="14.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="D3" s="16">
+      <c r="D3" s="14">
         <v>7</v>
       </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="17"/>
+      <c r="A4" s="15"/>
       <c r="B4" s="7"/>
       <c r="C4" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D4" s="18">
+      <c r="D4" s="16">
         <v>6</v>
       </c>
     </row>
     <row r="5" ht="14.25">
-      <c r="A5" s="17"/>
+      <c r="A5" s="15"/>
       <c r="B5" s="7"/>
       <c r="C5" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="16">
         <v>5</v>
       </c>
     </row>
     <row r="6" ht="14.25">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="15" t="s">
         <v>57</v>
       </c>
       <c r="B6" s="7" t="s">
@@ -1901,12 +2021,12 @@
       <c r="C6" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="16">
         <v>4</v>
       </c>
     </row>
     <row r="7" ht="14.25">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="15" t="s">
         <v>59</v>
       </c>
       <c r="B7" s="7" t="s">
@@ -1915,501 +2035,501 @@
       <c r="C7" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="16">
         <v>3</v>
       </c>
     </row>
     <row r="8" ht="14.25">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="17" t="s">
         <v>63</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="16">
         <v>2</v>
       </c>
     </row>
     <row r="9" ht="14.25">
-      <c r="A9" s="21"/>
-      <c r="B9" s="22"/>
-      <c r="C9" s="22" t="s">
+      <c r="A9" s="18"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="20">
         <v>1</v>
       </c>
     </row>
     <row r="13" ht="14.25">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="11" t="s">
+      <c r="C13" s="21"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="G13" s="24"/>
-      <c r="H13" s="11" t="s">
+      <c r="G13" s="21"/>
+      <c r="H13" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="I13" s="11"/>
-      <c r="J13" s="24" t="s">
+      <c r="I13" s="9"/>
+      <c r="J13" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="K13" s="24"/>
-      <c r="L13" s="25" t="s">
+      <c r="K13" s="21"/>
+      <c r="L13" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="M13" s="26"/>
-      <c r="N13" s="26"/>
-      <c r="O13" s="26"/>
-      <c r="P13" s="26"/>
+      <c r="M13" s="21"/>
+      <c r="N13" s="21"/>
+      <c r="O13" s="21"/>
+      <c r="P13" s="21"/>
     </row>
     <row r="14" ht="14.25">
-      <c r="A14" s="24"/>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="24"/>
-      <c r="K14" s="24"/>
-      <c r="L14" s="26"/>
-      <c r="M14" s="26"/>
-      <c r="N14" s="26"/>
-      <c r="O14" s="26"/>
-      <c r="P14" s="26"/>
+      <c r="A14" s="21"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="21"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="21"/>
+      <c r="K14" s="21"/>
+      <c r="L14" s="21"/>
+      <c r="M14" s="21"/>
+      <c r="N14" s="21"/>
+      <c r="O14" s="21"/>
+      <c r="P14" s="21"/>
     </row>
     <row r="15" ht="14.25">
-      <c r="A15" s="24"/>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="24"/>
-      <c r="K15" s="24"/>
-      <c r="L15" s="26"/>
-      <c r="M15" s="26"/>
-      <c r="N15" s="26"/>
-      <c r="O15" s="26"/>
-      <c r="P15" s="26"/>
+      <c r="A15" s="21"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="21"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="21"/>
+      <c r="K15" s="21"/>
+      <c r="L15" s="21"/>
+      <c r="M15" s="21"/>
+      <c r="N15" s="21"/>
+      <c r="O15" s="21"/>
+      <c r="P15" s="21"/>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="24"/>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="24"/>
-      <c r="K16" s="24"/>
-      <c r="L16" s="26"/>
-      <c r="M16" s="26"/>
-      <c r="N16" s="26"/>
-      <c r="O16" s="26"/>
-      <c r="P16" s="26"/>
+      <c r="A16" s="21"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="21"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="21"/>
+      <c r="K16" s="21"/>
+      <c r="L16" s="21"/>
+      <c r="M16" s="21"/>
+      <c r="N16" s="21"/>
+      <c r="O16" s="21"/>
+      <c r="P16" s="21"/>
     </row>
     <row r="17" ht="14.25">
-      <c r="A17" s="24" t="s">
+      <c r="A17" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="11" t="s">
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="G17" s="11"/>
-      <c r="H17" s="25" t="s">
+      <c r="G17" s="9"/>
+      <c r="H17" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="I17" s="11" t="s">
+      <c r="I17" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="J17" s="27" t="s">
+      <c r="J17" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="K17" s="26"/>
-      <c r="L17" s="25" t="s">
+      <c r="K17" s="21"/>
+      <c r="L17" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="M17" s="26"/>
-      <c r="N17" s="26"/>
-      <c r="O17" s="26"/>
-      <c r="P17" s="26"/>
+      <c r="M17" s="21"/>
+      <c r="N17" s="21"/>
+      <c r="O17" s="21"/>
+      <c r="P17" s="21"/>
     </row>
     <row r="18" ht="14.25">
-      <c r="A18" s="24"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="26"/>
-      <c r="K18" s="26"/>
-      <c r="L18" s="26"/>
-      <c r="M18" s="26"/>
-      <c r="N18" s="26"/>
-      <c r="O18" s="26"/>
-      <c r="P18" s="26"/>
+      <c r="A18" s="21"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="21"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="21"/>
+      <c r="P18" s="21"/>
     </row>
     <row r="19" ht="14.25">
-      <c r="A19" s="24"/>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="26"/>
-      <c r="K19" s="26"/>
-      <c r="L19" s="26"/>
-      <c r="M19" s="26"/>
-      <c r="N19" s="26"/>
-      <c r="O19" s="26"/>
-      <c r="P19" s="26"/>
+      <c r="A19" s="21"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="21"/>
+      <c r="K19" s="21"/>
+      <c r="L19" s="21"/>
+      <c r="M19" s="21"/>
+      <c r="N19" s="21"/>
+      <c r="O19" s="21"/>
+      <c r="P19" s="21"/>
     </row>
     <row r="20" ht="14.25">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="B20" s="27" t="s">
+      <c r="B20" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="C20" s="26"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="25" t="s">
+      <c r="C20" s="21"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G20" s="26"/>
-      <c r="H20" s="25" t="s">
+      <c r="G20" s="21"/>
+      <c r="H20" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="I20" s="25" t="s">
+      <c r="I20" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="J20" s="27" t="s">
+      <c r="J20" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="K20" s="26"/>
-      <c r="L20" s="25" t="s">
+      <c r="K20" s="21"/>
+      <c r="L20" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="M20" s="26"/>
-      <c r="N20" s="26"/>
-      <c r="O20" s="26"/>
-      <c r="P20" s="26"/>
+      <c r="M20" s="21"/>
+      <c r="N20" s="21"/>
+      <c r="O20" s="21"/>
+      <c r="P20" s="21"/>
     </row>
     <row r="21" ht="31.5" customHeight="1">
-      <c r="A21" s="26"/>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="26"/>
-      <c r="I21" s="26"/>
-      <c r="J21" s="26"/>
-      <c r="K21" s="26"/>
-      <c r="L21" s="26"/>
-      <c r="M21" s="26"/>
-      <c r="N21" s="26"/>
-      <c r="O21" s="26"/>
-      <c r="P21" s="26"/>
+      <c r="A21" s="21"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="21"/>
+      <c r="H21" s="21"/>
+      <c r="I21" s="21"/>
+      <c r="J21" s="21"/>
+      <c r="K21" s="21"/>
+      <c r="L21" s="21"/>
+      <c r="M21" s="21"/>
+      <c r="N21" s="21"/>
+      <c r="O21" s="21"/>
+      <c r="P21" s="21"/>
     </row>
     <row r="22" ht="14.25">
-      <c r="A22" s="27" t="s">
+      <c r="A22" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B22" s="27" t="s">
+      <c r="B22" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="25" t="s">
+      <c r="C22" s="21"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="G22" s="26"/>
-      <c r="H22" s="28" t="s">
+      <c r="G22" s="21"/>
+      <c r="H22" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="I22" s="25" t="s">
+      <c r="I22" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="J22" s="25" t="s">
+      <c r="J22" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="K22" s="26"/>
-      <c r="L22" s="25" t="s">
+      <c r="K22" s="21"/>
+      <c r="L22" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="M22" s="26"/>
-      <c r="N22" s="26"/>
-      <c r="O22" s="26"/>
-      <c r="P22" s="26"/>
+      <c r="M22" s="21"/>
+      <c r="N22" s="21"/>
+      <c r="O22" s="21"/>
+      <c r="P22" s="21"/>
     </row>
     <row r="23" ht="14.25">
-      <c r="A23" s="26"/>
-      <c r="B23" s="26"/>
-      <c r="C23" s="26"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="26"/>
-      <c r="J23" s="26"/>
-      <c r="K23" s="26"/>
-      <c r="L23" s="26"/>
-      <c r="M23" s="26"/>
-      <c r="N23" s="26"/>
-      <c r="O23" s="26"/>
-      <c r="P23" s="26"/>
+      <c r="A23" s="21"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="21"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="21"/>
+      <c r="J23" s="21"/>
+      <c r="K23" s="21"/>
+      <c r="L23" s="21"/>
+      <c r="M23" s="21"/>
+      <c r="N23" s="21"/>
+      <c r="O23" s="21"/>
+      <c r="P23" s="21"/>
     </row>
     <row r="24" ht="29.25" customHeight="1">
-      <c r="A24" s="26"/>
-      <c r="B24" s="26"/>
-      <c r="C24" s="26"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="26"/>
-      <c r="F24" s="26"/>
-      <c r="G24" s="26"/>
-      <c r="H24" s="28"/>
-      <c r="I24" s="26"/>
-      <c r="J24" s="26"/>
-      <c r="K24" s="26"/>
-      <c r="L24" s="26"/>
-      <c r="M24" s="26"/>
-      <c r="N24" s="26"/>
-      <c r="O24" s="26"/>
-      <c r="P24" s="26"/>
+      <c r="A24" s="21"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="21"/>
+      <c r="J24" s="21"/>
+      <c r="K24" s="21"/>
+      <c r="L24" s="21"/>
+      <c r="M24" s="21"/>
+      <c r="N24" s="21"/>
+      <c r="O24" s="21"/>
+      <c r="P24" s="21"/>
     </row>
     <row r="25" ht="14.25">
-      <c r="A25" s="24" t="s">
+      <c r="A25" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="B25" s="25" t="s">
+      <c r="B25" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="29"/>
-      <c r="F25" s="25" t="s">
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="G25" s="26"/>
-      <c r="H25" s="25" t="s">
+      <c r="G25" s="21"/>
+      <c r="H25" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="I25" s="26"/>
-      <c r="J25" s="27" t="s">
+      <c r="I25" s="21"/>
+      <c r="J25" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="K25" s="26"/>
-      <c r="L25" s="25" t="s">
+      <c r="K25" s="21"/>
+      <c r="L25" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="M25" s="26"/>
-      <c r="N25" s="26"/>
-      <c r="O25" s="26"/>
-      <c r="P25" s="26"/>
+      <c r="M25" s="21"/>
+      <c r="N25" s="21"/>
+      <c r="O25" s="21"/>
+      <c r="P25" s="21"/>
     </row>
     <row r="26" ht="14.25">
-      <c r="A26" s="24"/>
-      <c r="B26" s="29"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="29"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="26"/>
-      <c r="H26" s="26"/>
-      <c r="I26" s="26"/>
-      <c r="J26" s="26"/>
-      <c r="K26" s="26"/>
-      <c r="L26" s="26"/>
-      <c r="M26" s="26"/>
-      <c r="N26" s="26"/>
-      <c r="O26" s="26"/>
-      <c r="P26" s="26"/>
+      <c r="A26" s="21"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="21"/>
+      <c r="J26" s="21"/>
+      <c r="K26" s="21"/>
+      <c r="L26" s="21"/>
+      <c r="M26" s="21"/>
+      <c r="N26" s="21"/>
+      <c r="O26" s="21"/>
+      <c r="P26" s="21"/>
     </row>
     <row r="27" ht="29.25" customHeight="1">
-      <c r="A27" s="24"/>
-      <c r="B27" s="29"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="26"/>
-      <c r="H27" s="26"/>
-      <c r="I27" s="26"/>
-      <c r="J27" s="26"/>
-      <c r="K27" s="26"/>
-      <c r="L27" s="26"/>
-      <c r="M27" s="26"/>
-      <c r="N27" s="26"/>
-      <c r="O27" s="26"/>
-      <c r="P27" s="26"/>
+      <c r="A27" s="21"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="21"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="21"/>
+      <c r="J27" s="21"/>
+      <c r="K27" s="21"/>
+      <c r="L27" s="21"/>
+      <c r="M27" s="21"/>
+      <c r="N27" s="21"/>
+      <c r="O27" s="21"/>
+      <c r="P27" s="21"/>
     </row>
     <row r="28" ht="14.25">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="B28" s="27" t="s">
+      <c r="B28" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="25" t="s">
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="G28" s="26"/>
-      <c r="H28" s="25" t="s">
+      <c r="G28" s="21"/>
+      <c r="H28" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="I28" s="26"/>
-      <c r="J28" s="27" t="s">
+      <c r="I28" s="21"/>
+      <c r="J28" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="K28" s="26"/>
-      <c r="L28" s="25" t="s">
+      <c r="K28" s="21"/>
+      <c r="L28" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="M28" s="26"/>
-      <c r="N28" s="26"/>
-      <c r="O28" s="26"/>
-      <c r="P28" s="26"/>
+      <c r="M28" s="21"/>
+      <c r="N28" s="21"/>
+      <c r="O28" s="21"/>
+      <c r="P28" s="21"/>
     </row>
     <row r="29" ht="14.25">
-      <c r="A29" s="24"/>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26"/>
-      <c r="H29" s="26"/>
-      <c r="I29" s="26"/>
-      <c r="J29" s="26"/>
-      <c r="K29" s="26"/>
-      <c r="L29" s="26"/>
-      <c r="M29" s="26"/>
-      <c r="N29" s="26"/>
-      <c r="O29" s="26"/>
-      <c r="P29" s="26"/>
+      <c r="A29" s="21"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="21"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="21"/>
+      <c r="G29" s="21"/>
+      <c r="H29" s="21"/>
+      <c r="I29" s="21"/>
+      <c r="J29" s="21"/>
+      <c r="K29" s="21"/>
+      <c r="L29" s="21"/>
+      <c r="M29" s="21"/>
+      <c r="N29" s="21"/>
+      <c r="O29" s="21"/>
+      <c r="P29" s="21"/>
     </row>
     <row r="30" ht="47.25" customHeight="1">
-      <c r="A30" s="24"/>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="26"/>
-      <c r="J30" s="26"/>
-      <c r="K30" s="26"/>
-      <c r="L30" s="26"/>
-      <c r="M30" s="26"/>
-      <c r="N30" s="26"/>
-      <c r="O30" s="26"/>
-      <c r="P30" s="26"/>
+      <c r="A30" s="21"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="21"/>
+      <c r="J30" s="21"/>
+      <c r="K30" s="21"/>
+      <c r="L30" s="21"/>
+      <c r="M30" s="21"/>
+      <c r="N30" s="21"/>
+      <c r="O30" s="21"/>
+      <c r="P30" s="21"/>
     </row>
     <row r="31" ht="14.25">
-      <c r="A31" s="27" t="s">
+      <c r="A31" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="B31" s="27" t="s">
+      <c r="B31" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="C31" s="26"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="25" t="s">
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="G31" s="26"/>
-      <c r="H31" s="25" t="s">
+      <c r="G31" s="21"/>
+      <c r="H31" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="I31" s="24"/>
-      <c r="J31" s="24" t="s">
+      <c r="I31" s="21"/>
+      <c r="J31" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="K31" s="30"/>
-      <c r="L31" s="25" t="s">
+      <c r="K31" s="21"/>
+      <c r="L31" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="M31" s="26"/>
-      <c r="N31" s="26"/>
-      <c r="O31" s="26"/>
-      <c r="P31" s="26"/>
+      <c r="M31" s="21"/>
+      <c r="N31" s="21"/>
+      <c r="O31" s="21"/>
+      <c r="P31" s="21"/>
     </row>
     <row r="32" ht="14.25">
-      <c r="A32" s="26"/>
-      <c r="B32" s="26"/>
-      <c r="C32" s="26"/>
-      <c r="D32" s="26"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="24"/>
-      <c r="J32" s="30"/>
-      <c r="K32" s="30"/>
-      <c r="L32" s="26"/>
-      <c r="M32" s="26"/>
-      <c r="N32" s="26"/>
-      <c r="O32" s="26"/>
-      <c r="P32" s="26"/>
+      <c r="A32" s="21"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="21"/>
+      <c r="K32" s="21"/>
+      <c r="L32" s="21"/>
+      <c r="M32" s="21"/>
+      <c r="N32" s="21"/>
+      <c r="O32" s="21"/>
+      <c r="P32" s="21"/>
     </row>
     <row r="33" ht="35.25" customHeight="1">
-      <c r="A33" s="26"/>
-      <c r="B33" s="26"/>
-      <c r="C33" s="26"/>
-      <c r="D33" s="26"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26"/>
-      <c r="I33" s="24"/>
-      <c r="J33" s="30"/>
-      <c r="K33" s="30"/>
-      <c r="L33" s="26"/>
-      <c r="M33" s="26"/>
-      <c r="N33" s="26"/>
-      <c r="O33" s="26"/>
-      <c r="P33" s="26"/>
+      <c r="A33" s="21"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="I33" s="21"/>
+      <c r="J33" s="21"/>
+      <c r="K33" s="21"/>
+      <c r="L33" s="21"/>
+      <c r="M33" s="21"/>
+      <c r="N33" s="21"/>
+      <c r="O33" s="21"/>
+      <c r="P33" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="53">
@@ -2473,4 +2593,227 @@
   <headerFooter/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="29.421875"/>
+    <col customWidth="1" min="2" max="2" width="39.8515625"/>
+    <col customWidth="1" min="3" max="3" width="13.140625"/>
+    <col customWidth="1" min="4" max="4" width="27.00390625"/>
+    <col customWidth="1" min="5" max="5" width="22.28125"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="37.5" customHeight="1">
+      <c r="A1" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="B1" s="22"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>131</v>
+      </c>
+      <c r="B10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>133</v>
+      </c>
+      <c r="B11" t="s">
+        <v>134</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>135</v>
+      </c>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>136</v>
+      </c>
+      <c r="B12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B13" t="s">
+        <v>139</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>142</v>
+      </c>
+      <c r="B16" t="s">
+        <v>143</v>
+      </c>
+      <c r="C16" s="26" t="s">
+        <v>144</v>
+      </c>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+    </row>
+    <row r="17" ht="15">
+      <c r="A17" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="B17" t="s">
+        <v>146</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>147</v>
+      </c>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+    </row>
+    <row r="18" ht="15">
+      <c r="A18" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="B18" t="s">
+        <v>149</v>
+      </c>
+      <c r="C18" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>151</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C17:E17"/>
+  </mergeCells>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Finished with M1.2 module. Added the files Configure VLAN and Trunk txt and cisco pkt. Also A small update on the cheat sheet on the cisco sheet.
</commit_message>
<xml_diff>
--- a/Cheat_Sheet_SecuritateIT.xlsx
+++ b/Cheat_Sheet_SecuritateIT.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="169">
   <si>
     <t xml:space="preserve">GitHub </t>
   </si>
@@ -529,6 +529,57 @@
   </si>
   <si>
     <t xml:space="preserve">SSH config</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uername name password parola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">creates user and password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">username admin password admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ip domain-name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set's the router domain name - used for SSH key generation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ip domain-name networking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">krypto key generate rsa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">generate RSA key for  SSH encryption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">krypto key nererate rsa then followed by the number of bytes 512 to 4000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ip ssh version 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enable SSH version</t>
+  </si>
+  <si>
+    <t xml:space="preserve">line vty 0 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allows for up to 5 simultaneous connection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">login local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authetnicate remote users using local username and password database</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transport input ssh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allows only SSH connection on VTY lines</t>
   </si>
 </sst>
 </file>
@@ -554,7 +605,6 @@
     </font>
     <font>
       <sz val="12.000000"/>
-      <color indexed="64"/>
       <name val="Times New Roman"/>
     </font>
   </fonts>
@@ -699,7 +749,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="26">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -763,15 +813,13 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -2597,13 +2645,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="29.421875"/>
-    <col customWidth="1" min="2" max="2" width="39.8515625"/>
+    <col customWidth="1" min="2" max="2" width="63.140625"/>
     <col customWidth="1" min="3" max="3" width="13.140625"/>
     <col customWidth="1" min="4" max="4" width="27.00390625"/>
-    <col customWidth="1" min="5" max="5" width="22.28125"/>
+    <col customWidth="1" min="5" max="5" width="24.140625"/>
   </cols>
   <sheetData>
     <row r="1" ht="37.5" customHeight="1">
@@ -2611,8 +2659,8 @@
         <v>110</v>
       </c>
       <c r="B1" s="22"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -2621,11 +2669,11 @@
       <c r="B2" t="s">
         <v>112</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -2650,10 +2698,10 @@
       <c r="E4" s="7"/>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="8" t="s">
         <v>119</v>
       </c>
       <c r="C5" s="7"/>
@@ -2667,7 +2715,7 @@
       <c r="B6" t="s">
         <v>121</v>
       </c>
-      <c r="C6" s="26" t="s">
+      <c r="C6" s="10" t="s">
         <v>122</v>
       </c>
       <c r="D6" s="10"/>
@@ -2680,7 +2728,7 @@
       <c r="B7" t="s">
         <v>124</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="C7" s="10" t="s">
         <v>125</v>
       </c>
       <c r="D7" s="10"/>
@@ -2701,11 +2749,11 @@
       <c r="B9" t="s">
         <v>129</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
@@ -2722,11 +2770,11 @@
       <c r="B11" t="s">
         <v>134</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="C11" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
@@ -2743,11 +2791,11 @@
       <c r="B13" t="s">
         <v>139</v>
       </c>
-      <c r="C13" s="24" t="s">
+      <c r="C13" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
@@ -2761,27 +2809,27 @@
       <c r="B16" t="s">
         <v>143</v>
       </c>
-      <c r="C16" s="26" t="s">
+      <c r="C16" s="10" t="s">
         <v>144</v>
       </c>
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
     </row>
     <row r="17" ht="15">
-      <c r="A17" s="27" t="s">
+      <c r="A17" s="23" t="s">
         <v>145</v>
       </c>
       <c r="B17" t="s">
         <v>146</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="C17" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
     </row>
     <row r="18" ht="15">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="23" t="s">
         <v>148</v>
       </c>
       <c r="B18" t="s">
@@ -2796,8 +2844,79 @@
         <v>151</v>
       </c>
     </row>
+    <row r="21" ht="14.25">
+      <c r="A21" t="s">
+        <v>152</v>
+      </c>
+      <c r="B21" t="s">
+        <v>153</v>
+      </c>
+      <c r="C21" s="24" t="s">
+        <v>154</v>
+      </c>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="A22" t="s">
+        <v>155</v>
+      </c>
+      <c r="B22" t="s">
+        <v>156</v>
+      </c>
+      <c r="C22" s="24" t="s">
+        <v>157</v>
+      </c>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+    </row>
+    <row r="23" ht="14.25">
+      <c r="A23" t="s">
+        <v>158</v>
+      </c>
+      <c r="B23" t="s">
+        <v>159</v>
+      </c>
+      <c r="C23" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="A24" t="s">
+        <v>161</v>
+      </c>
+      <c r="B24" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="A25" t="s">
+        <v>163</v>
+      </c>
+      <c r="B25" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="A26" t="s">
+        <v>165</v>
+      </c>
+      <c r="B26" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="27" ht="14.25">
+      <c r="A27" t="s">
+        <v>167</v>
+      </c>
+      <c r="B27" t="s">
+        <v>168</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="15">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="C3:E3"/>
@@ -2810,6 +2929,9 @@
     <mergeCell ref="C13:E13"/>
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="C23:E23"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>